<commit_message>
change TC-AM-02-UI-02 into pass
</commit_message>
<xml_diff>
--- a/docs/test/test-cases/Test case Authentication Module Register-Login.xlsx
+++ b/docs/test/test-cases/Test case Authentication Module Register-Login.xlsx
@@ -14,10 +14,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="198">
   <si>
-    <t>Project: Recall AI</t>
+    <t>Function/Feature ID</t>
   </si>
   <si>
-    <t>Function/Feature ID</t>
+    <t>Project: Recall AI</t>
   </si>
   <si>
     <t>Case ID</t>
@@ -103,7 +103,16 @@
     <t>TC-AM-01-02</t>
   </si>
   <si>
+    <t>Register account</t>
+  </si>
+  <si>
     <t>Register fails when email already exists</t>
+  </si>
+  <si>
+    <t>Allows new users to create a personal account in the system by submitting required registration details, including full name, email address, and a secure password.</t>
+  </si>
+  <si>
+    <t>Requires email uniqueness across the platform. Passwords must comply with minimum security requirements (at least 8 characters). Upon successful registration, the system automatically logs the user in and redirects them to the main dashboard.</t>
   </si>
   <si>
     <t>1. Open Postman, create request POST /api/v1/auth/register.
@@ -121,16 +130,7 @@
 - No new record is created in the DB</t>
   </si>
   <si>
-    <t>Register account</t>
-  </si>
-  <si>
-    <t>Allows new users to create a personal account in the system by submitting required registration details, including full name, email address, and a secure password.</t>
-  </si>
-  <si>
     <t>HTTP 409 Conflict. success: false. error.code: "EMAIL_CONFLICT". error.message describes the existing email error. No duplicate record created in DB.</t>
-  </si>
-  <si>
-    <t>Requires email uniqueness across the platform. Passwords must comply with minimum security requirements (at least 8 characters). Upon successful registration, the system automatically logs the user in and redirects them to the main dashboard.</t>
   </si>
   <si>
     <t>Important: also check the DB to confirm no duplicate record was created.</t>
@@ -750,10 +750,11 @@
 - Deny access to the Dashboard</t>
   </si>
   <si>
-    <t>Sign In button changes to loading state (spinner) and hangs indefinitely, system does not display the "Email or password incorrect" error message nor does it release the button's loading state.</t>
+    <t>- Display error message: "Email or password incorrect"
+- Stay in login page</t>
   </si>
   <si>
-    <t>BUG: The Sign In button gets stuck in an infinite loading state</t>
+    <t>Displayed error message is identical → specific cause is not revealed (User Enumeration prevention).</t>
   </si>
   <si>
     <t>TC-AM-02-UI-03</t>
@@ -814,14 +815,14 @@
     </font>
     <font>
       <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <color theme="1"/>
-      <name val="Arial"/>
     </font>
     <font>
       <color theme="1"/>
@@ -921,21 +922,21 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -953,7 +954,7 @@
     <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -1185,12 +1186,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+      <c r="A1" s="2" t="s">
+        <v>1</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
@@ -1215,12 +1216,12 @@
       <c r="Z1" s="5"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
@@ -1245,10 +1246,10 @@
       <c r="Z2" s="5"/>
     </row>
     <row r="3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -1273,10 +1274,10 @@
       <c r="Z3" s="5"/>
     </row>
     <row r="4">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
@@ -1301,16 +1302,16 @@
       <c r="Z4" s="5"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="5"/>
@@ -1341,13 +1342,13 @@
         <v>13</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -29237,34 +29238,34 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>10</v>
       </c>
       <c r="K1" s="5"/>
@@ -29361,16 +29362,16 @@
         <v>25</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>19</v>
@@ -30551,8 +30552,8 @@
       <c r="F29" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="G29" s="11" t="s">
-        <v>74</v>
+      <c r="G29" s="8" t="s">
+        <v>19</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Pass TC-AM-01-08: dont allow password with only 'space'
</commit_message>
<xml_diff>
--- a/docs/test/test-cases/Test case Authentication Module Register-Login.xlsx
+++ b/docs/test/test-cases/Test case Authentication Module Register-Login.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="197">
   <si>
     <t>Function/Feature ID</t>
   </si>
@@ -59,6 +59,15 @@
     <t>TC-AM-01-01</t>
   </si>
   <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Feature Name</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
     <t>Register successfully with valid data</t>
   </si>
   <si>
@@ -85,34 +94,37 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>NMPhat</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Feature Name</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Main happy path. If this TC fails, other UC-01 TCs may not run.</t>
-  </si>
-  <si>
-    <t>TC-AM-01-02</t>
-  </si>
-  <si>
     <t>Register account</t>
-  </si>
-  <si>
-    <t>Register fails when email already exists</t>
   </si>
   <si>
     <t>Allows new users to create a personal account in the system by submitting required registration details, including full name, email address, and a secure password.</t>
   </si>
   <si>
     <t>Requires email uniqueness across the platform. Passwords must comply with minimum security requirements (at least 8 characters). Upon successful registration, the system automatically logs the user in and redirects them to the main dashboard.</t>
+  </si>
+  <si>
+    <t>NMPhat</t>
+  </si>
+  <si>
+    <t>UC-02</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Enables existing registered users to authenticate into the system using their registered email and password to access protected features and personal data</t>
+  </si>
+  <si>
+    <t>Main happy path. If this TC fails, other UC-01 TCs may not run.</t>
+  </si>
+  <si>
+    <t>Displays generic error messages (e.g., 'Invalid email or password') upon authentication failure to prevent user enumeration. Supports session persistence and automatic token renewal.</t>
+  </si>
+  <si>
+    <t>TC-AM-01-02</t>
+  </si>
+  <si>
+    <t>Register fails when email already exists</t>
   </si>
   <si>
     <t>1. Open Postman, create request POST /api/v1/auth/register.
@@ -134,18 +146,6 @@
   </si>
   <si>
     <t>Important: also check the DB to confirm no duplicate record was created.</t>
-  </si>
-  <si>
-    <t>UC-02</t>
-  </si>
-  <si>
-    <t>Login</t>
-  </si>
-  <si>
-    <t>Enables existing registered users to authenticate into the system using their registered email and password to access protected features and personal data</t>
-  </si>
-  <si>
-    <t>Displays generic error messages (e.g., 'Invalid email or password') upon authentication failure to prevent user enumeration. Supports session persistence and automatic token renewal.</t>
   </si>
   <si>
     <t>TC-AM-01-03</t>
@@ -307,13 +307,10 @@
     <t>- HTTP Status: 400 Bad Request (should be rejected for security reasons)</t>
   </si>
   <si>
-    <t>HTTP 201 Created. The server accepted an all-whitespace password and created the account successfully. This is a security bug that must be fixed on the backend.</t>
+    <t xml:space="preserve">HTTP 400 Bad Request. The server rejects requests with whitespace-only passwords and returns a validation error.   </t>
   </si>
   <si>
-    <t>Fail - Bug</t>
-  </si>
-  <si>
-    <t>BUG: Zod schema is missing .trim().min(8) or .refine(v =&gt; v.trim().length &gt;= 8) to reject whitespace-only passwords. A trim() rule needs to be added to the validator.</t>
+    <t xml:space="preserve">Zod validator successfully rejects whitespace-only passwords using `trim()` / whitespace validation. </t>
   </si>
   <si>
     <t>TC-AM-01-UI-01</t>
@@ -835,7 +832,7 @@
     </font>
     <font/>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -852,12 +849,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
         <bgColor rgb="FFE2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4E4"/>
-        <bgColor rgb="FFFCE4E4"/>
       </patternFill>
     </fill>
     <fill>
@@ -917,7 +908,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -942,19 +933,16 @@
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -1303,13 +1291,13 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>10</v>
@@ -1338,17 +1326,17 @@
       <c r="Z5" s="5"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>26</v>
+      <c r="B6" s="8" t="s">
+        <v>23</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>28</v>
+      <c r="C6" s="8" t="s">
+        <v>24</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>29</v>
+      <c r="D6" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -1374,17 +1362,17 @@
       <c r="Z6" s="5"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="s">
-        <v>34</v>
+      <c r="A7" s="8" t="s">
+        <v>27</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>35</v>
+      <c r="B7" s="8" t="s">
+        <v>28</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>36</v>
+      <c r="C7" s="8" t="s">
+        <v>29</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>37</v>
+      <c r="D7" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
@@ -29314,28 +29302,28 @@
         <v>14</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
-      <c r="G3" s="8" t="s">
-        <v>19</v>
+      <c r="G3" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="10">
         <v>46227.0</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
@@ -29359,31 +29347,31 @@
         <v>13</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
-      <c r="G4" s="8" t="s">
-        <v>19</v>
+      <c r="G4" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="10">
         <v>46227.0</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K4" s="5"/>
       <c r="L4" s="5"/>
@@ -29421,13 +29409,13 @@
       <c r="F5" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="G5" s="8" t="s">
-        <v>19</v>
+      <c r="G5" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="10">
         <v>46227.0</v>
       </c>
       <c r="J5" s="7" t="s">
@@ -29469,13 +29457,13 @@
       <c r="F6" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="9" t="s">
         <v>49</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="10">
         <v>46227.0</v>
       </c>
       <c r="J6" s="7" t="s">
@@ -29517,13 +29505,13 @@
       <c r="F7" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="9" t="s">
         <v>49</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="10">
         <v>46227.0</v>
       </c>
       <c r="J7" s="7" t="s">
@@ -29565,13 +29553,13 @@
       <c r="F8" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G8" s="8" t="s">
-        <v>19</v>
+      <c r="G8" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="10">
         <v>46227.0</v>
       </c>
       <c r="J8" s="7" t="s">
@@ -29613,13 +29601,13 @@
       <c r="F9" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="8" t="s">
-        <v>19</v>
+      <c r="G9" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="10">
         <v>46227.0</v>
       </c>
       <c r="J9" s="7" t="s">
@@ -29661,17 +29649,17 @@
       <c r="F10" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="G10" s="11" t="s">
-        <v>74</v>
+      <c r="G10" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I10" s="9">
-        <v>46227.0</v>
+      <c r="I10" s="10">
+        <v>46232.0</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
@@ -29694,32 +29682,32 @@
       <c r="A11" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="D11" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="E11" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="F11" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>19</v>
+      <c r="G11" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="10">
         <v>46227.0</v>
       </c>
-      <c r="J11" s="10" t="s">
-        <v>81</v>
+      <c r="J11" s="8" t="s">
+        <v>80</v>
       </c>
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
@@ -29741,32 +29729,32 @@
       <c r="A12" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="D12" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="E12" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="F12" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>19</v>
+      <c r="G12" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I12" s="9">
+      <c r="I12" s="10">
         <v>46227.0</v>
       </c>
-      <c r="J12" s="10" t="s">
-        <v>87</v>
+      <c r="J12" s="8" t="s">
+        <v>86</v>
       </c>
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
@@ -29789,32 +29777,32 @@
       <c r="A13" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="D13" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="E13" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="F13" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>19</v>
+      <c r="G13" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="10">
         <v>46227.0</v>
       </c>
-      <c r="J13" s="10" t="s">
-        <v>93</v>
+      <c r="J13" s="8" t="s">
+        <v>92</v>
       </c>
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
@@ -29837,32 +29825,32 @@
       <c r="A14" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="D14" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="E14" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="F14" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>19</v>
+      <c r="G14" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I14" s="9">
+      <c r="I14" s="10">
         <v>46227.0</v>
       </c>
-      <c r="J14" s="10" t="s">
-        <v>99</v>
+      <c r="J14" s="8" t="s">
+        <v>98</v>
       </c>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
@@ -29885,32 +29873,32 @@
       <c r="A15" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="D15" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="E15" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="F15" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="F15" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>19</v>
+      <c r="G15" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I15" s="9">
+      <c r="I15" s="10">
         <v>46227.0</v>
       </c>
-      <c r="J15" s="10" t="s">
-        <v>105</v>
+      <c r="J15" s="8" t="s">
+        <v>104</v>
       </c>
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
@@ -29933,32 +29921,32 @@
       <c r="A16" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="D16" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="E16" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="F16" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>19</v>
+      <c r="G16" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="10">
         <v>46227.0</v>
       </c>
-      <c r="J16" s="10" t="s">
-        <v>111</v>
+      <c r="J16" s="8" t="s">
+        <v>110</v>
       </c>
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
@@ -29978,18 +29966,18 @@
       <c r="Z16" s="5"/>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="s">
-        <v>112</v>
+      <c r="A17" s="11" t="s">
+        <v>111</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="14"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="13"/>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
@@ -30009,34 +29997,34 @@
     </row>
     <row r="18">
       <c r="A18" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="E18" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="F18" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>19</v>
+      <c r="G18" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I18" s="9">
+      <c r="I18" s="10">
         <v>46227.0</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
@@ -30057,34 +30045,34 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B19" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="E19" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="F19" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>19</v>
+      <c r="G19" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I19" s="9">
+      <c r="I19" s="10">
         <v>46227.0</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
@@ -30105,34 +30093,34 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="D20" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="E20" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="F20" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="F20" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>19</v>
+      <c r="G20" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I20" s="9">
+      <c r="I20" s="10">
         <v>46227.0</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
@@ -30153,34 +30141,34 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B21" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="E21" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="F21" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="F21" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>19</v>
+      <c r="G21" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I21" s="9">
+      <c r="I21" s="10">
         <v>46227.0</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
@@ -30201,34 +30189,34 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B22" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="D22" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="E22" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="F22" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>19</v>
+      <c r="G22" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I22" s="9">
+      <c r="I22" s="10">
         <v>46227.0</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
@@ -30249,30 +30237,30 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B23" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C23" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="D23" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="E23" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="F23" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="G23" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="G23" s="8" t="s">
-        <v>148</v>
+      <c r="H23" s="7" t="s">
+        <v>26</v>
       </c>
-      <c r="H23" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I23" s="9">
+      <c r="I23" s="10">
         <v>46227.0</v>
       </c>
       <c r="J23" s="7"/>
@@ -30295,34 +30283,34 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="D24" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="E24" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="F24" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="F24" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>19</v>
+      <c r="G24" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I24" s="9">
+      <c r="I24" s="10">
         <v>46227.0</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
@@ -30343,34 +30331,34 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="E25" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="F25" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="F25" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>19</v>
+      <c r="G25" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I25" s="9">
+      <c r="I25" s="10">
         <v>46227.0</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
@@ -30391,34 +30379,34 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B26" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="D26" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="E26" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="F26" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="G26" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="G26" s="8" t="s">
-        <v>166</v>
+      <c r="H26" s="7" t="s">
+        <v>26</v>
       </c>
-      <c r="H26" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I26" s="9">
+      <c r="I26" s="10">
         <v>46227.0</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
@@ -30439,34 +30427,34 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B27" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="D27" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="E27" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="F27" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="F27" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>148</v>
+      <c r="G27" s="9" t="s">
+        <v>147</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I27" s="9">
+      <c r="I27" s="10">
         <v>46227.0</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K27" s="5"/>
       <c r="L27" s="5"/>
@@ -30487,34 +30475,34 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B28" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C28" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="D28" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="E28" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="F28" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="F28" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>19</v>
+      <c r="G28" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I28" s="9">
+      <c r="I28" s="10">
         <v>46227.0</v>
       </c>
-      <c r="J28" s="10" t="s">
-        <v>179</v>
+      <c r="J28" s="8" t="s">
+        <v>178</v>
       </c>
       <c r="K28" s="5"/>
       <c r="L28" s="5"/>
@@ -30535,34 +30523,34 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B29" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C29" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="D29" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="E29" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="F29" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="F29" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>19</v>
+      <c r="G29" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I29" s="9">
+      <c r="I29" s="10">
         <v>46227.0</v>
       </c>
-      <c r="J29" s="10" t="s">
-        <v>185</v>
+      <c r="J29" s="8" t="s">
+        <v>184</v>
       </c>
       <c r="K29" s="5"/>
       <c r="L29" s="5"/>
@@ -30583,34 +30571,34 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B30" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C30" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="D30" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="E30" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="F30" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="F30" s="10" t="s">
-        <v>190</v>
-      </c>
-      <c r="G30" s="8" t="s">
-        <v>19</v>
+      <c r="G30" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I30" s="9">
+      <c r="I30" s="10">
         <v>46227.0</v>
       </c>
-      <c r="J30" s="10" t="s">
-        <v>191</v>
+      <c r="J30" s="8" t="s">
+        <v>190</v>
       </c>
       <c r="K30" s="5"/>
       <c r="L30" s="5"/>
@@ -30631,34 +30619,34 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="C31" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="D31" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="E31" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="F31" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="F31" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="G31" s="8" t="s">
-        <v>19</v>
+      <c r="G31" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
-      <c r="I31" s="9">
+      <c r="I31" s="10">
         <v>46227.0</v>
       </c>
-      <c r="J31" s="10" t="s">
-        <v>197</v>
+      <c r="J31" s="8" t="s">
+        <v>196</v>
       </c>
       <c r="K31" s="5"/>
       <c r="L31" s="5"/>

</xml_diff>